<commit_message>
docs: wbs 수정본 xlsx, pdf 업로드
</commit_message>
<xml_diff>
--- a/docs/requirements/요구사항_정의서.xlsx
+++ b/docs/requirements/요구사항_정의서.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bini/Desktop/Bini/단위프로젝트/SKN30-FINAL-5Team/docs/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D879FEBF-FB06-5542-8CD8-062DC36CE8EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8BE52D0-33C1-EC4E-8E0B-34C9F2B9A58B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,9 @@
     <sheet name="핵심 요구사항 요약" sheetId="1" r:id="rId1"/>
     <sheet name="상세 목록" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'핵심 요구사항 요약'!$A$1:$G$62</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -5154,29 +5157,11 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5217,9 +5202,6 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5237,12 +5219,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="12" fillId="9" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5262,12 +5238,6 @@
     <xf numFmtId="3" fontId="12" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="14" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5283,12 +5253,6 @@
     <xf numFmtId="3" fontId="12" fillId="6" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="15" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="16" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5303,6 +5267,45 @@
     </xf>
     <xf numFmtId="3" fontId="12" fillId="7" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="15" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5530,1006 +5533,1006 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="73" t="s">
         <v>1595</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1">
-      <c r="A3" s="32"/>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
+      <c r="A3" s="27"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
     </row>
     <row r="4" spans="1:7" ht="25" customHeight="1">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="33" t="s">
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="33"/>
+      <c r="G4" s="74"/>
     </row>
     <row r="5" spans="1:7" ht="25" customHeight="1">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="32"/>
-      <c r="F5" s="34" t="s">
+      <c r="E5" s="27"/>
+      <c r="F5" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="35" t="s">
+      <c r="G5" s="29" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="25" customHeight="1">
-      <c r="A6" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="36">
+      <c r="A6" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="30">
         <v>193</v>
       </c>
-      <c r="C6" s="36" t="s">
+      <c r="C6" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="37" t="s">
+      <c r="D6" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="32"/>
-      <c r="F6" s="36" t="s">
+      <c r="E6" s="27"/>
+      <c r="F6" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="38" t="s">
+      <c r="G6" s="32" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="25" customHeight="1">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="39">
+      <c r="B7" s="33">
         <v>114</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="32"/>
-      <c r="F7" s="41" t="s">
+      <c r="E7" s="27"/>
+      <c r="F7" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="38" t="s">
+      <c r="G7" s="32" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="25" customHeight="1">
-      <c r="A8" s="42" t="s">
+      <c r="A8" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="42">
+      <c r="B8" s="36">
         <v>65</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="43" t="s">
+      <c r="D8" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
     </row>
     <row r="9" spans="1:7" ht="25" customHeight="1">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="41">
+      <c r="B9" s="35">
         <v>75</v>
       </c>
-      <c r="C9" s="41" t="s">
+      <c r="C9" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="44" t="s">
+      <c r="D9" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
     </row>
     <row r="10" spans="1:7" ht="25" customHeight="1">
-      <c r="A10" s="45" t="s">
+      <c r="A10" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="45">
+      <c r="B10" s="39">
         <v>447</v>
       </c>
-      <c r="C10" s="45" t="s">
+      <c r="C10" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="46" t="s">
+      <c r="D10" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="32"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
     </row>
     <row r="11" spans="1:7" ht="15" customHeight="1">
-      <c r="A11" s="32"/>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
+      <c r="A11" s="27"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1">
-      <c r="A12" s="32"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
+      <c r="A12" s="27"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
     </row>
     <row r="13" spans="1:7" ht="20" customHeight="1">
-      <c r="A13" s="47" t="s">
+      <c r="A13" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="47"/>
-      <c r="C13" s="47"/>
-      <c r="D13" s="47"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
+      <c r="B13" s="75"/>
+      <c r="C13" s="75"/>
+      <c r="D13" s="75"/>
+      <c r="E13" s="75"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
     </row>
     <row r="14" spans="1:7" ht="20" customHeight="1">
-      <c r="A14" s="34" t="s">
+      <c r="A14" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="34" t="s">
+      <c r="B14" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="34" t="s">
+      <c r="C14" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="34" t="s">
+      <c r="D14" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="E14" s="34" t="s">
+      <c r="E14" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
     </row>
     <row r="15" spans="1:7" ht="20" customHeight="1">
-      <c r="A15" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" s="48" t="s">
+      <c r="A15" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="49">
+      <c r="C15" s="42">
         <v>5</v>
       </c>
-      <c r="D15" s="50" t="s">
+      <c r="D15" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="50" t="s">
+      <c r="E15" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="F15" s="32"/>
-      <c r="G15" s="32"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
     </row>
     <row r="16" spans="1:7" ht="20" customHeight="1">
-      <c r="A16" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B16" s="48" t="s">
+      <c r="A16" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="49">
+      <c r="C16" s="42">
         <v>14</v>
       </c>
-      <c r="D16" s="50" t="s">
+      <c r="D16" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="50" t="s">
+      <c r="E16" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
     </row>
     <row r="17" spans="1:7" ht="20" customHeight="1">
-      <c r="A17" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17" s="48" t="s">
+      <c r="A17" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="49">
+      <c r="C17" s="42">
         <v>20</v>
       </c>
-      <c r="D17" s="50" t="s">
+      <c r="D17" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="50" t="s">
+      <c r="E17" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
     </row>
     <row r="18" spans="1:7" ht="20" customHeight="1">
-      <c r="A18" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" s="48" t="s">
+      <c r="A18" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="49">
+      <c r="C18" s="42">
         <v>8</v>
       </c>
-      <c r="D18" s="50" t="s">
+      <c r="D18" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="50" t="s">
+      <c r="E18" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
     </row>
     <row r="19" spans="1:7" ht="20" customHeight="1">
-      <c r="A19" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19" s="48" t="s">
+      <c r="A19" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="49">
+      <c r="C19" s="42">
         <v>77</v>
       </c>
-      <c r="D19" s="50" t="s">
+      <c r="D19" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="50" t="s">
+      <c r="E19" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
     </row>
     <row r="20" spans="1:7" ht="20" customHeight="1">
-      <c r="A20" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" s="48" t="s">
+      <c r="A20" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="49">
+      <c r="C20" s="42">
         <v>14</v>
       </c>
-      <c r="D20" s="50" t="s">
+      <c r="D20" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="50" t="s">
+      <c r="E20" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
     </row>
     <row r="21" spans="1:7" ht="20" customHeight="1">
-      <c r="A21" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B21" s="48" t="s">
+      <c r="A21" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="49">
-        <v>9</v>
-      </c>
-      <c r="D21" s="50" t="s">
+      <c r="C21" s="42">
+        <v>9</v>
+      </c>
+      <c r="D21" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="50" t="s">
+      <c r="E21" s="43" t="s">
         <v>52</v>
       </c>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
     </row>
     <row r="22" spans="1:7" ht="20" customHeight="1">
-      <c r="A22" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B22" s="48" t="s">
+      <c r="A22" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="41" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="49">
+      <c r="C22" s="42">
         <v>21</v>
       </c>
-      <c r="D22" s="50" t="s">
+      <c r="D22" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="E22" s="50" t="s">
+      <c r="E22" s="43" t="s">
         <v>55</v>
       </c>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
     </row>
     <row r="23" spans="1:7" ht="20" customHeight="1">
-      <c r="A23" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" s="48" t="s">
+      <c r="A23" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="49">
+      <c r="C23" s="42">
         <v>10</v>
       </c>
-      <c r="D23" s="50" t="s">
+      <c r="D23" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="E23" s="50" t="s">
+      <c r="E23" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
     </row>
     <row r="24" spans="1:7" ht="20" customHeight="1">
-      <c r="A24" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24" s="48" t="s">
+      <c r="A24" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="41" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="49">
+      <c r="C24" s="42">
         <v>15</v>
       </c>
-      <c r="D24" s="50" t="s">
+      <c r="D24" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="E24" s="50" t="s">
+      <c r="E24" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
     </row>
     <row r="25" spans="1:7" ht="20" customHeight="1">
-      <c r="A25" s="51" t="s">
+      <c r="A25" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="51"/>
-      <c r="C25" s="52">
+      <c r="B25" s="44"/>
+      <c r="C25" s="45">
         <v>193</v>
       </c>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
     </row>
     <row r="26" spans="1:7" ht="20" customHeight="1">
-      <c r="A26" s="32"/>
-      <c r="B26" s="32"/>
-      <c r="C26" s="53"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
+      <c r="A26" s="27"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
     </row>
     <row r="27" spans="1:7" ht="20" customHeight="1">
-      <c r="A27" s="54" t="s">
+      <c r="A27" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="B27" s="54"/>
-      <c r="C27" s="55"/>
-      <c r="D27" s="54"/>
-      <c r="E27" s="54"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
+      <c r="B27" s="66"/>
+      <c r="C27" s="67"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="66"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
     </row>
     <row r="28" spans="1:7" ht="20" customHeight="1">
-      <c r="A28" s="34" t="s">
+      <c r="A28" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="34" t="s">
+      <c r="B28" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="56" t="s">
+      <c r="C28" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="34" t="s">
+      <c r="D28" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="E28" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
     </row>
     <row r="29" spans="1:7" ht="20" customHeight="1">
-      <c r="A29" s="57" t="s">
+      <c r="A29" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B29" s="57" t="s">
+      <c r="B29" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="58">
+      <c r="C29" s="49">
         <v>7</v>
       </c>
-      <c r="D29" s="59" t="s">
+      <c r="D29" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="59" t="s">
+      <c r="E29" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="F29" s="32"/>
-      <c r="G29" s="32"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
     </row>
     <row r="30" spans="1:7" ht="20" customHeight="1">
-      <c r="A30" s="57" t="s">
+      <c r="A30" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B30" s="57" t="s">
+      <c r="B30" s="48" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="58">
+      <c r="C30" s="49">
         <v>12</v>
       </c>
-      <c r="D30" s="59" t="s">
+      <c r="D30" s="50" t="s">
         <v>67</v>
       </c>
-      <c r="E30" s="59" t="s">
+      <c r="E30" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
     </row>
     <row r="31" spans="1:7" ht="20" customHeight="1">
-      <c r="A31" s="57" t="s">
+      <c r="A31" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B31" s="57" t="s">
+      <c r="B31" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="58">
+      <c r="C31" s="49">
         <v>23</v>
       </c>
-      <c r="D31" s="59" t="s">
+      <c r="D31" s="50" t="s">
         <v>68</v>
       </c>
-      <c r="E31" s="59" t="s">
+      <c r="E31" s="50" t="s">
         <v>52</v>
       </c>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
     </row>
     <row r="32" spans="1:7" ht="20" customHeight="1">
-      <c r="A32" s="57" t="s">
+      <c r="A32" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B32" s="57" t="s">
+      <c r="B32" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="C32" s="58">
+      <c r="C32" s="49">
         <v>7</v>
       </c>
-      <c r="D32" s="59" t="s">
+      <c r="D32" s="50" t="s">
         <v>69</v>
       </c>
-      <c r="E32" s="59" t="s">
+      <c r="E32" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="F32" s="32"/>
-      <c r="G32" s="32"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
     </row>
     <row r="33" spans="1:7" ht="20" customHeight="1">
-      <c r="A33" s="57" t="s">
+      <c r="A33" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="57" t="s">
+      <c r="B33" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="C33" s="58">
+      <c r="C33" s="49">
         <v>29</v>
       </c>
-      <c r="D33" s="59" t="s">
+      <c r="D33" s="50" t="s">
         <v>71</v>
       </c>
-      <c r="E33" s="59" t="s">
+      <c r="E33" s="50" t="s">
         <v>72</v>
       </c>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
     </row>
     <row r="34" spans="1:7" ht="20" customHeight="1">
-      <c r="A34" s="57" t="s">
+      <c r="A34" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B34" s="57" t="s">
+      <c r="B34" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="58">
+      <c r="C34" s="49">
         <v>16</v>
       </c>
-      <c r="D34" s="59" t="s">
+      <c r="D34" s="50" t="s">
         <v>73</v>
       </c>
-      <c r="E34" s="59" t="s">
+      <c r="E34" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
     </row>
     <row r="35" spans="1:7" ht="20" customHeight="1">
-      <c r="A35" s="57" t="s">
+      <c r="A35" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="57" t="s">
+      <c r="B35" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="58">
+      <c r="C35" s="49">
         <v>8</v>
       </c>
-      <c r="D35" s="59" t="s">
+      <c r="D35" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="E35" s="59" t="s">
+      <c r="E35" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
     </row>
     <row r="36" spans="1:7" ht="20" customHeight="1">
-      <c r="A36" s="57" t="s">
+      <c r="A36" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="57" t="s">
+      <c r="B36" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="C36" s="58">
+      <c r="C36" s="49">
         <v>6</v>
       </c>
-      <c r="D36" s="59" t="s">
+      <c r="D36" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="E36" s="59" t="s">
+      <c r="E36" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
     </row>
     <row r="37" spans="1:7" ht="20" customHeight="1">
-      <c r="A37" s="57" t="s">
+      <c r="A37" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B37" s="57" t="s">
+      <c r="B37" s="48" t="s">
         <v>80</v>
       </c>
-      <c r="C37" s="58">
+      <c r="C37" s="49">
         <v>6</v>
       </c>
-      <c r="D37" s="59" t="s">
+      <c r="D37" s="50" t="s">
         <v>81</v>
       </c>
-      <c r="E37" s="59" t="s">
+      <c r="E37" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
     </row>
     <row r="38" spans="1:7" ht="20" customHeight="1">
-      <c r="A38" s="60" t="s">
+      <c r="A38" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="B38" s="60"/>
-      <c r="C38" s="61">
+      <c r="B38" s="51"/>
+      <c r="C38" s="52">
         <v>114</v>
       </c>
-      <c r="D38" s="60"/>
-      <c r="E38" s="60"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
+      <c r="D38" s="51"/>
+      <c r="E38" s="51"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
     </row>
     <row r="39" spans="1:7" ht="20" customHeight="1">
-      <c r="A39" s="32"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="53"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
+      <c r="A39" s="27"/>
+      <c r="B39" s="27"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="27"/>
+      <c r="G39" s="27"/>
     </row>
     <row r="40" spans="1:7" ht="20" customHeight="1">
-      <c r="A40" s="62" t="s">
+      <c r="A40" s="68" t="s">
         <v>84</v>
       </c>
-      <c r="B40" s="62"/>
-      <c r="C40" s="63"/>
-      <c r="D40" s="62"/>
-      <c r="E40" s="62"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
+      <c r="B40" s="68"/>
+      <c r="C40" s="69"/>
+      <c r="D40" s="68"/>
+      <c r="E40" s="68"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
     </row>
     <row r="41" spans="1:7" ht="20" customHeight="1">
-      <c r="A41" s="34" t="s">
+      <c r="A41" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B41" s="34" t="s">
+      <c r="B41" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C41" s="56" t="s">
+      <c r="C41" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="D41" s="34" t="s">
+      <c r="D41" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="E41" s="34" t="s">
+      <c r="E41" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="F41" s="32"/>
-      <c r="G41" s="32"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
     </row>
     <row r="42" spans="1:7" ht="20" customHeight="1">
-      <c r="A42" s="64" t="s">
+      <c r="A42" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="B42" s="64" t="s">
+      <c r="B42" s="53" t="s">
         <v>85</v>
       </c>
-      <c r="C42" s="65">
+      <c r="C42" s="54">
         <v>6</v>
       </c>
-      <c r="D42" s="66" t="s">
+      <c r="D42" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="E42" s="66" t="s">
+      <c r="E42" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
+      <c r="F42" s="27"/>
+      <c r="G42" s="27"/>
     </row>
     <row r="43" spans="1:7" ht="20" customHeight="1">
-      <c r="A43" s="64" t="s">
+      <c r="A43" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="B43" s="64" t="s">
+      <c r="B43" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="C43" s="65">
+      <c r="C43" s="54">
         <v>16</v>
       </c>
-      <c r="D43" s="66" t="s">
+      <c r="D43" s="55" t="s">
         <v>89</v>
       </c>
-      <c r="E43" s="66" t="s">
+      <c r="E43" s="55" t="s">
         <v>90</v>
       </c>
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="27"/>
     </row>
     <row r="44" spans="1:7" ht="20" customHeight="1">
-      <c r="A44" s="64" t="s">
+      <c r="A44" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="B44" s="64" t="s">
+      <c r="B44" s="53" t="s">
         <v>91</v>
       </c>
-      <c r="C44" s="65">
+      <c r="C44" s="54">
         <v>14</v>
       </c>
-      <c r="D44" s="66" t="s">
+      <c r="D44" s="55" t="s">
         <v>92</v>
       </c>
-      <c r="E44" s="66" t="s">
+      <c r="E44" s="55" t="s">
         <v>93</v>
       </c>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
+      <c r="F44" s="27"/>
+      <c r="G44" s="27"/>
     </row>
     <row r="45" spans="1:7" ht="20" customHeight="1">
-      <c r="A45" s="64" t="s">
+      <c r="A45" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="B45" s="64" t="s">
+      <c r="B45" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="C45" s="65">
+      <c r="C45" s="54">
         <v>7</v>
       </c>
-      <c r="D45" s="66" t="s">
+      <c r="D45" s="55" t="s">
         <v>94</v>
       </c>
-      <c r="E45" s="66" t="s">
+      <c r="E45" s="55" t="s">
         <v>76</v>
       </c>
-      <c r="F45" s="32"/>
-      <c r="G45" s="32"/>
+      <c r="F45" s="27"/>
+      <c r="G45" s="27"/>
     </row>
     <row r="46" spans="1:7" ht="20" customHeight="1">
-      <c r="A46" s="64" t="s">
+      <c r="A46" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="B46" s="64" t="s">
+      <c r="B46" s="53" t="s">
         <v>95</v>
       </c>
-      <c r="C46" s="65">
+      <c r="C46" s="54">
         <v>6</v>
       </c>
-      <c r="D46" s="66" t="s">
+      <c r="D46" s="55" t="s">
         <v>96</v>
       </c>
-      <c r="E46" s="66" t="s">
+      <c r="E46" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="F46" s="32"/>
-      <c r="G46" s="32"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
     </row>
     <row r="47" spans="1:7" ht="20" customHeight="1">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="64" t="s">
+      <c r="B47" s="53" t="s">
         <v>98</v>
       </c>
-      <c r="C47" s="65">
+      <c r="C47" s="54">
         <v>16</v>
       </c>
-      <c r="D47" s="66" t="s">
+      <c r="D47" s="55" t="s">
         <v>99</v>
       </c>
-      <c r="E47" s="66" t="s">
+      <c r="E47" s="55" t="s">
         <v>100</v>
       </c>
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
+      <c r="F47" s="27"/>
+      <c r="G47" s="27"/>
     </row>
     <row r="48" spans="1:7" ht="20" customHeight="1">
-      <c r="A48" s="67" t="s">
+      <c r="A48" s="56" t="s">
         <v>101</v>
       </c>
-      <c r="B48" s="67"/>
-      <c r="C48" s="68">
+      <c r="B48" s="56"/>
+      <c r="C48" s="57">
         <v>65</v>
       </c>
-      <c r="D48" s="67"/>
-      <c r="E48" s="67"/>
-      <c r="F48" s="32"/>
-      <c r="G48" s="32"/>
+      <c r="D48" s="56"/>
+      <c r="E48" s="56"/>
+      <c r="F48" s="27"/>
+      <c r="G48" s="27"/>
     </row>
     <row r="49" spans="1:7" ht="20" customHeight="1">
-      <c r="A49" s="32"/>
-      <c r="B49" s="32"/>
-      <c r="C49" s="53"/>
-      <c r="D49" s="32"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="32"/>
-      <c r="G49" s="32"/>
+      <c r="A49" s="27"/>
+      <c r="B49" s="27"/>
+      <c r="C49" s="46"/>
+      <c r="D49" s="27"/>
+      <c r="E49" s="27"/>
+      <c r="F49" s="27"/>
+      <c r="G49" s="27"/>
     </row>
     <row r="50" spans="1:7" ht="20" customHeight="1">
-      <c r="A50" s="69" t="s">
+      <c r="A50" s="70" t="s">
         <v>102</v>
       </c>
-      <c r="B50" s="69"/>
-      <c r="C50" s="70"/>
-      <c r="D50" s="69"/>
-      <c r="E50" s="69"/>
-      <c r="F50" s="32"/>
-      <c r="G50" s="32"/>
+      <c r="B50" s="70"/>
+      <c r="C50" s="71"/>
+      <c r="D50" s="70"/>
+      <c r="E50" s="70"/>
+      <c r="F50" s="27"/>
+      <c r="G50" s="27"/>
     </row>
     <row r="51" spans="1:7" ht="20" customHeight="1">
-      <c r="A51" s="34" t="s">
+      <c r="A51" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B51" s="34" t="s">
+      <c r="B51" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C51" s="56" t="s">
+      <c r="C51" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="D51" s="34" t="s">
+      <c r="D51" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="E51" s="34" t="s">
+      <c r="E51" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="F51" s="32"/>
-      <c r="G51" s="32"/>
+      <c r="F51" s="27"/>
+      <c r="G51" s="27"/>
     </row>
     <row r="52" spans="1:7" ht="20" customHeight="1">
-      <c r="A52" s="71" t="s">
+      <c r="A52" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B52" s="71" t="s">
+      <c r="B52" s="58" t="s">
         <v>103</v>
       </c>
-      <c r="C52" s="72">
+      <c r="C52" s="59">
         <v>8</v>
       </c>
-      <c r="D52" s="73" t="s">
+      <c r="D52" s="60" t="s">
         <v>104</v>
       </c>
-      <c r="E52" s="73" t="s">
+      <c r="E52" s="60" t="s">
         <v>105</v>
       </c>
-      <c r="F52" s="32"/>
-      <c r="G52" s="32"/>
+      <c r="F52" s="27"/>
+      <c r="G52" s="27"/>
     </row>
     <row r="53" spans="1:7" ht="20" customHeight="1">
-      <c r="A53" s="71" t="s">
+      <c r="A53" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B53" s="71" t="s">
+      <c r="B53" s="58" t="s">
         <v>106</v>
       </c>
-      <c r="C53" s="72">
+      <c r="C53" s="59">
         <v>6</v>
       </c>
-      <c r="D53" s="73" t="s">
+      <c r="D53" s="60" t="s">
         <v>107</v>
       </c>
-      <c r="E53" s="73" t="s">
+      <c r="E53" s="60" t="s">
         <v>108</v>
       </c>
-      <c r="F53" s="32"/>
-      <c r="G53" s="32"/>
+      <c r="F53" s="27"/>
+      <c r="G53" s="27"/>
     </row>
     <row r="54" spans="1:7" ht="20" customHeight="1">
-      <c r="A54" s="71" t="s">
+      <c r="A54" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B54" s="71" t="s">
+      <c r="B54" s="58" t="s">
         <v>109</v>
       </c>
-      <c r="C54" s="72">
+      <c r="C54" s="59">
         <v>15</v>
       </c>
-      <c r="D54" s="73" t="s">
+      <c r="D54" s="60" t="s">
         <v>110</v>
       </c>
-      <c r="E54" s="73" t="s">
+      <c r="E54" s="60" t="s">
         <v>111</v>
       </c>
-      <c r="F54" s="32"/>
-      <c r="G54" s="32"/>
+      <c r="F54" s="27"/>
+      <c r="G54" s="27"/>
     </row>
     <row r="55" spans="1:7" ht="20" customHeight="1">
-      <c r="A55" s="71" t="s">
+      <c r="A55" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B55" s="71" t="s">
+      <c r="B55" s="58" t="s">
         <v>112</v>
       </c>
-      <c r="C55" s="72">
+      <c r="C55" s="59">
         <v>10</v>
       </c>
-      <c r="D55" s="73" t="s">
+      <c r="D55" s="60" t="s">
         <v>113</v>
       </c>
-      <c r="E55" s="73" t="s">
+      <c r="E55" s="60" t="s">
         <v>114</v>
       </c>
-      <c r="F55" s="32"/>
-      <c r="G55" s="32"/>
+      <c r="F55" s="27"/>
+      <c r="G55" s="27"/>
     </row>
     <row r="56" spans="1:7" ht="20" customHeight="1">
-      <c r="A56" s="71" t="s">
+      <c r="A56" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B56" s="71" t="s">
+      <c r="B56" s="58" t="s">
         <v>115</v>
       </c>
-      <c r="C56" s="72">
+      <c r="C56" s="59">
         <v>7</v>
       </c>
-      <c r="D56" s="73" t="s">
+      <c r="D56" s="60" t="s">
         <v>116</v>
       </c>
-      <c r="E56" s="73" t="s">
+      <c r="E56" s="60" t="s">
         <v>117</v>
       </c>
-      <c r="F56" s="32"/>
-      <c r="G56" s="32"/>
+      <c r="F56" s="27"/>
+      <c r="G56" s="27"/>
     </row>
     <row r="57" spans="1:7" ht="20" customHeight="1">
-      <c r="A57" s="71" t="s">
+      <c r="A57" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B57" s="71" t="s">
+      <c r="B57" s="58" t="s">
         <v>118</v>
       </c>
-      <c r="C57" s="72">
+      <c r="C57" s="59">
         <v>11</v>
       </c>
-      <c r="D57" s="73" t="s">
+      <c r="D57" s="60" t="s">
         <v>119</v>
       </c>
-      <c r="E57" s="73" t="s">
+      <c r="E57" s="60" t="s">
         <v>120</v>
       </c>
-      <c r="F57" s="32"/>
-      <c r="G57" s="32"/>
+      <c r="F57" s="27"/>
+      <c r="G57" s="27"/>
     </row>
     <row r="58" spans="1:7" ht="20" customHeight="1">
-      <c r="A58" s="71" t="s">
+      <c r="A58" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B58" s="71" t="s">
+      <c r="B58" s="58" t="s">
         <v>121</v>
       </c>
-      <c r="C58" s="72">
+      <c r="C58" s="59">
         <v>11</v>
       </c>
-      <c r="D58" s="73" t="s">
+      <c r="D58" s="60" t="s">
         <v>122</v>
       </c>
-      <c r="E58" s="73" t="s">
+      <c r="E58" s="60" t="s">
         <v>123</v>
       </c>
-      <c r="F58" s="32"/>
-      <c r="G58" s="32"/>
+      <c r="F58" s="27"/>
+      <c r="G58" s="27"/>
     </row>
     <row r="59" spans="1:7" ht="20" customHeight="1">
-      <c r="A59" s="71" t="s">
+      <c r="A59" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B59" s="71" t="s">
+      <c r="B59" s="58" t="s">
         <v>124</v>
       </c>
-      <c r="C59" s="72">
+      <c r="C59" s="59">
         <v>7</v>
       </c>
-      <c r="D59" s="73" t="s">
+      <c r="D59" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="E59" s="73" t="s">
+      <c r="E59" s="60" t="s">
         <v>126</v>
       </c>
-      <c r="F59" s="32"/>
-      <c r="G59" s="32"/>
+      <c r="F59" s="27"/>
+      <c r="G59" s="27"/>
     </row>
     <row r="60" spans="1:7" ht="20" customHeight="1">
-      <c r="A60" s="74" t="s">
+      <c r="A60" s="61" t="s">
         <v>127</v>
       </c>
-      <c r="B60" s="74"/>
-      <c r="C60" s="75">
+      <c r="B60" s="61"/>
+      <c r="C60" s="62">
         <v>75</v>
       </c>
-      <c r="D60" s="74"/>
-      <c r="E60" s="74"/>
-      <c r="F60" s="32"/>
-      <c r="G60" s="32"/>
+      <c r="D60" s="61"/>
+      <c r="E60" s="61"/>
+      <c r="F60" s="27"/>
+      <c r="G60" s="27"/>
     </row>
     <row r="61" spans="1:7" ht="15">
       <c r="A61" s="6"/>
@@ -7551,7 +7554,8 @@
     <mergeCell ref="A13:E13"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="37" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -7569,60 +7573,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="40" customHeight="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="63" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
     </row>
     <row r="2" spans="1:7" ht="15">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="64" t="s">
         <v>129</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
     </row>
     <row r="3" spans="1:7" ht="15">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="65" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="65" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28" t="s">
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65" t="s">
         <v>132</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="65" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16">
-      <c r="A4" s="28"/>
-      <c r="B4" s="29" t="s">
+      <c r="A4" s="65"/>
+      <c r="B4" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="E4" s="29" t="s">
+      <c r="E4" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
     </row>
     <row r="5" spans="1:7" s="6" customFormat="1" ht="28" customHeight="1">
       <c r="A5" s="1" t="s">

</xml_diff>